<commit_message>
fixde run tm robot dynamics program error
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/ur_dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/ur_dynamics_calc.xlsx
@@ -450,19 +450,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20.57045398965127</v>
+        <v>1.244139824930656e-30</v>
       </c>
       <c r="B2" t="n">
-        <v>236.2713165154749</v>
+        <v>80.04971379600001</v>
       </c>
       <c r="C2" t="n">
-        <v>89.95618028252025</v>
+        <v>21.91520646</v>
       </c>
       <c r="D2" t="n">
-        <v>2.608345354344999</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>-3.091636386906274</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>